<commit_message>
data: benchmark n=20 completo — 15/15 estrategias×casos, φ exacto
- 5 estrategias × 3 casos: todas convergen al mismo φ que QNodos
- IB: ×28 (caso 1), ×53 (caso 2), ×47 (caso 3) más rápido que QNodos
- Particiones reales guardadas en resultado_20A.json y DatosML2026.xlsx 20A-Elementos
- QNodos referencia: 26899s / 10712s / 11263s vs IB: 960s / 201s / 239s
</commit_message>
<xml_diff>
--- a/DatosML2026.xlsx
+++ b/DatosML2026.xlsx
@@ -5574,35 +5574,59 @@
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>(ver benchmark)</t>
+          <t>(M=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 18, 19)) | (M*=(), A*=(17,))</t>
         </is>
       </c>
       <c r="E7" s="18" t="n">
         <v>0.023633</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>2350.3</v>
+        <v>2243.1</v>
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>(ver benchmark)</t>
+          <t>(M=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 18, 19)) | (M*=(), A*=(17,))</t>
         </is>
       </c>
       <c r="H7" s="19" t="n">
         <v>0.023633</v>
       </c>
       <c r="I7" s="19" t="n">
-        <v>1310.4</v>
-      </c>
-      <c r="J7" s="20" t="n"/>
-      <c r="K7" s="20" t="n"/>
-      <c r="L7" s="20" t="n"/>
-      <c r="M7" s="21" t="n"/>
-      <c r="N7" s="21" t="n"/>
-      <c r="O7" s="21" t="n"/>
-      <c r="P7" s="22" t="n"/>
-      <c r="Q7" s="22" t="n"/>
-      <c r="R7" s="22" t="n"/>
+        <v>960.5</v>
+      </c>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t>(M=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 18, 19)) | (M*=(), A*=(17,))</t>
+        </is>
+      </c>
+      <c r="K7" s="20" t="n">
+        <v>0.023633</v>
+      </c>
+      <c r="L7" s="20" t="n">
+        <v>1880.6</v>
+      </c>
+      <c r="M7" s="21" t="inlineStr">
+        <is>
+          <t>(M=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 18, 19)) | (M*=(), A*=(17,))</t>
+        </is>
+      </c>
+      <c r="N7" s="21" t="n">
+        <v>0.023633</v>
+      </c>
+      <c r="O7" s="21" t="n">
+        <v>1754.3</v>
+      </c>
+      <c r="P7" s="22" t="inlineStr">
+        <is>
+          <t>(M=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 18, 19)) | (M*=(), A*=(17,))</t>
+        </is>
+      </c>
+      <c r="Q7" s="22" t="n">
+        <v>0.023633</v>
+      </c>
+      <c r="R7" s="22" t="n">
+        <v>2760.5</v>
+      </c>
       <c r="S7" s="18" t="n"/>
       <c r="T7" s="18" t="n"/>
       <c r="U7" s="18" t="n"/>
@@ -5676,75 +5700,59 @@
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E8" s="25" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F8" s="25" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>(M=(), A=(7,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18), A*=(0, 1, 2, 3, 4, 5, 6, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19))</t>
+        </is>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>0.02621</v>
+      </c>
+      <c r="F8" s="25" t="n">
+        <v>667.9</v>
       </c>
       <c r="G8" s="26" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H8" s="27" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I8" s="27" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>(M=(), A=(7,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18), A*=(0, 1, 2, 3, 4, 5, 6, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19))</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="n">
+        <v>0.02621</v>
+      </c>
+      <c r="I8" s="27" t="n">
+        <v>201.6</v>
       </c>
       <c r="J8" s="28" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K8" s="29" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L8" s="29" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>(M=(), A=(7,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18), A*=(0, 1, 2, 3, 4, 5, 6, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19))</t>
+        </is>
+      </c>
+      <c r="K8" s="29" t="n">
+        <v>0.02621</v>
+      </c>
+      <c r="L8" s="29" t="n">
+        <v>697.2</v>
       </c>
       <c r="M8" s="30" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N8" s="31" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O8" s="31" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>(M=(), A=(7,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18), A*=(0, 1, 2, 3, 4, 5, 6, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19))</t>
+        </is>
+      </c>
+      <c r="N8" s="31" t="n">
+        <v>0.02621</v>
+      </c>
+      <c r="O8" s="31" t="n">
+        <v>661.3</v>
       </c>
       <c r="P8" s="32" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q8" s="33" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R8" s="33" t="n"/>
+          <t>(M=(), A=(7,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18), A*=(0, 1, 2, 3, 4, 5, 6, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19))</t>
+        </is>
+      </c>
+      <c r="Q8" s="33" t="n">
+        <v>0.02621</v>
+      </c>
+      <c r="R8" s="33" t="n">
+        <v>1383.5</v>
+      </c>
       <c r="S8" s="24" t="n"/>
       <c r="T8" s="25" t="n"/>
       <c r="U8" s="25" t="n"/>
@@ -5818,75 +5826,59 @@
       </c>
       <c r="D9" s="24" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E9" s="25" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F9" s="25" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>(M=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 14, 15, 16, 17, 18, 19)) | (M*=(), A*=(13,))</t>
+        </is>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>0.019691</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>692</v>
       </c>
       <c r="G9" s="26" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H9" s="27" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I9" s="27" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>(M=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 14, 15, 16, 17, 18, 19)) | (M*=(), A*=(13,))</t>
+        </is>
+      </c>
+      <c r="H9" s="27" t="n">
+        <v>0.019691</v>
+      </c>
+      <c r="I9" s="27" t="n">
+        <v>239</v>
       </c>
       <c r="J9" s="28" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K9" s="29" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L9" s="29" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>(M=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 14, 15, 16, 17, 18, 19)) | (M*=(), A*=(13,))</t>
+        </is>
+      </c>
+      <c r="K9" s="29" t="n">
+        <v>0.019691</v>
+      </c>
+      <c r="L9" s="29" t="n">
+        <v>753.6</v>
       </c>
       <c r="M9" s="30" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N9" s="31" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O9" s="31" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>(M=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 14, 15, 16, 17, 18, 19)) | (M*=(), A*=(13,))</t>
+        </is>
+      </c>
+      <c r="N9" s="31" t="n">
+        <v>0.019691</v>
+      </c>
+      <c r="O9" s="31" t="n">
+        <v>717.3</v>
       </c>
       <c r="P9" s="32" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Q9" s="33" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R9" s="33" t="n"/>
+          <t>(M=(), A=(13,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 14, 15, 16, 17, 18, 19))</t>
+        </is>
+      </c>
+      <c r="Q9" s="33" t="n">
+        <v>0.019691</v>
+      </c>
+      <c r="R9" s="33" t="n">
+        <v>1917</v>
+      </c>
       <c r="S9" s="24" t="n"/>
       <c r="T9" s="25" t="n"/>
       <c r="U9" s="25" t="n"/>

</xml_diff>

<commit_message>
feat: IBQNodos ×290-385 más rápido que QNodos en n=20, φ exacto
- Corrige bug k_bipartir → bipartir en _evaluar_asig para k=2
- Agrega multi-start paralelo con ThreadPoolExecutor
- n=20 caso 1: IBQNodos 92s vs IB 803s vs QNodos 26899s
- README y DatosML2026.xlsx actualizados con tabla comparativa
</commit_message>
<xml_diff>
--- a/DatosML2026.xlsx
+++ b/DatosML2026.xlsx
@@ -147,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -250,6 +250,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5395,9 +5401,9 @@
           <t>k = 2</t>
         </is>
       </c>
-      <c r="S5" s="9" t="inlineStr">
-        <is>
-          <t>k = 3</t>
+      <c r="S5" s="36" t="inlineStr">
+        <is>
+          <t>IBQNodos</t>
         </is>
       </c>
       <c r="AH5" s="10" t="inlineStr">
@@ -5452,9 +5458,19 @@
           <t>REMCMC</t>
         </is>
       </c>
-      <c r="S6" s="12" t="inlineStr">
-        <is>
-          <t>Louvain</t>
+      <c r="S6" s="37" t="inlineStr">
+        <is>
+          <t>Partición</t>
+        </is>
+      </c>
+      <c r="T6" s="35" t="inlineStr">
+        <is>
+          <t>Pérdida</t>
+        </is>
+      </c>
+      <c r="U6" s="35" t="inlineStr">
+        <is>
+          <t>Tiempo (s)</t>
         </is>
       </c>
       <c r="V6" s="13" t="inlineStr">
@@ -5627,9 +5643,17 @@
       <c r="R7" s="22" t="n">
         <v>2760.5</v>
       </c>
-      <c r="S7" s="18" t="n"/>
-      <c r="T7" s="18" t="n"/>
-      <c r="U7" s="18" t="n"/>
+      <c r="S7" s="18" t="inlineStr">
+        <is>
+          <t>(M=(), A=(17,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 18, 19))</t>
+        </is>
+      </c>
+      <c r="T7" s="18" t="n">
+        <v>0.023633</v>
+      </c>
+      <c r="U7" s="18" t="n">
+        <v>92.90000000000001</v>
+      </c>
       <c r="V7" s="19" t="n"/>
       <c r="W7" s="19" t="n"/>
       <c r="X7" s="19" t="n"/>
@@ -5753,9 +5777,17 @@
       <c r="R8" s="33" t="n">
         <v>1383.5</v>
       </c>
-      <c r="S8" s="24" t="n"/>
-      <c r="T8" s="25" t="n"/>
-      <c r="U8" s="25" t="n"/>
+      <c r="S8" s="24" t="inlineStr">
+        <is>
+          <t>(M=(), A=(7,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18), A*=(0, 1, 2, 3, 4, 5, 6, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19))</t>
+        </is>
+      </c>
+      <c r="T8" s="25" t="n">
+        <v>0.02621</v>
+      </c>
+      <c r="U8" s="25" t="n">
+        <v>27.8</v>
+      </c>
       <c r="V8" s="26" t="n"/>
       <c r="W8" s="27" t="n"/>
       <c r="X8" s="27" t="n"/>
@@ -5879,9 +5911,17 @@
       <c r="R9" s="33" t="n">
         <v>1917</v>
       </c>
-      <c r="S9" s="24" t="n"/>
-      <c r="T9" s="25" t="n"/>
-      <c r="U9" s="25" t="n"/>
+      <c r="S9" s="24" t="inlineStr">
+        <is>
+          <t>(M=(), A=(13,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19), A*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 14, 15, 16, 17, 18, 19))</t>
+        </is>
+      </c>
+      <c r="T9" s="25" t="n">
+        <v>0.019691</v>
+      </c>
+      <c r="U9" s="25" t="n">
+        <v>30.6</v>
+      </c>
       <c r="V9" s="26" t="n"/>
       <c r="W9" s="27" t="n"/>
       <c r="X9" s="27" t="n"/>
@@ -6000,7 +6040,7 @@
       <c r="BK10" s="33" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="27">
     <mergeCell ref="BQ4:BS4"/>
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="G6:I6"/>
@@ -6009,15 +6049,14 @@
     <mergeCell ref="AW5:BK5"/>
     <mergeCell ref="V6:X6"/>
     <mergeCell ref="AH6:AJ6"/>
-    <mergeCell ref="S6:U6"/>
     <mergeCell ref="Y6:AA6"/>
     <mergeCell ref="BI6:BK6"/>
     <mergeCell ref="BM5:BO5"/>
     <mergeCell ref="AE6:AG6"/>
     <mergeCell ref="AK6:AM6"/>
     <mergeCell ref="BM4:BO4"/>
+    <mergeCell ref="S5:U5"/>
     <mergeCell ref="AQ6:AS6"/>
-    <mergeCell ref="S5:AG5"/>
     <mergeCell ref="D5:R5"/>
     <mergeCell ref="AB6:AD6"/>
     <mergeCell ref="BC6:BE6"/>

</xml_diff>